<commit_message>
Tableau E5 : documents/productions précis, croix multiples justifiées
</commit_message>
<xml_diff>
--- a/assets/Tableau_E5_Kabir_AMOUSSA.xlsx
+++ b/assets/Tableau_E5_Kabir_AMOUSSA.xlsx
@@ -1385,14 +1385,18 @@
     <row r="9" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Administration Active Directory (TP TRANSCUBE) : groupes de sécurité, partage RH sécurisé (permissions NTFS), stratégies de mot de passe/verrouillage, quotas disque.</t>
+          <t>Administration Active Directory — TP TRANSCUBE (groupes, GPO, quotas). Documents : capture des groupes de sécurité et des permissions NTFS du partage RH, export des stratégies de groupe (mot de passe, verrouillage), paramétrage des quotas disque.</t>
         </is>
       </c>
       <c r="B9" s="11" t="n"/>
       <c r="C9" s="18" t="n"/>
       <c r="D9" s="21" t="n"/>
       <c r="E9" s="21" t="n"/>
-      <c r="F9" s="21" t="n"/>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
           <t>X</t>
@@ -1403,7 +1407,7 @@
     <row r="10" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>VLAN, routage inter-VLAN et VTP (Packet Tracer) : configuration des VLAN, routage par sous-interfaces, déploiement automatisé via VTP.</t>
+          <t>VLAN, routage inter-VLAN et VTP — Exolab Packet Tracer. Documents : maquette Packet Tracer (.pkt), captures des trames étiquetées 802.1Q et de la configuration VTP (serveur/clients).</t>
         </is>
       </c>
       <c r="B10" s="11" t="n"/>
@@ -1415,13 +1419,17 @@
       <c r="D10" s="21" t="n"/>
       <c r="E10" s="21" t="n"/>
       <c r="F10" s="21" t="n"/>
-      <c r="G10" s="21" t="n"/>
+      <c r="G10" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H10" s="22" t="n"/>
     </row>
     <row r="11" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Service DHCP/DNS et extension réseau (plan d'action en équipe) : mise en service DHCP/DNS, raccordement d'un nouveau bureau (switch, PC, imprimante).</t>
+          <t>Service DHCP/DNS et extension réseau — plan d'action en équipe. Documents : plan d'action rédigé, maquette Packet Tracer, captures des baux DHCP et des enregistrements DNS.</t>
         </is>
       </c>
       <c r="B11" s="11" t="n"/>
@@ -1433,17 +1441,25 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G11" s="21" t="n"/>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H11" s="22" t="n"/>
     </row>
     <row r="12" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Virtualisation et PowerShell (plan d'action en équipe) : création/clonage de 2 VM Windows 10, administration en réseau interne (renommage, adressage IP).</t>
+          <t>Virtualisation et administration PowerShell — plan d'action en équipe. Documents : plan d'action rédigé, captures des commandes PowerShell (Rename-Computer, New-NetIPAddress) et des tests de connectivité.</t>
         </is>
       </c>
       <c r="B12" s="11" t="n"/>
-      <c r="C12" s="21" t="n"/>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D12" s="21" t="n"/>
       <c r="E12" s="21" t="n"/>
       <c r="F12" s="21" t="inlineStr">
@@ -1457,7 +1473,7 @@
     <row r="13" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Prise en main de PowerShell : cmdlets de base (Get-Process, Get-Service, Where-Object, New-Item), premier script avec variables.</t>
+          <t>Prise en main de PowerShell. Documents : tableau des commandes testées, captures des résultats, premier script PowerShell ISE.</t>
         </is>
       </c>
       <c r="B13" s="11" t="n"/>
@@ -1473,24 +1489,40 @@
       </c>
     </row>
     <row r="14" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A14" s="13" t="n"/>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Création et mise à jour du portfolio numérique. Documents : site publié en ligne (akabir-07.github.io), code source (HTML/CSS/JS) versionné sur GitHub.</t>
+        </is>
+      </c>
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="21" t="n"/>
       <c r="D14" s="21" t="n"/>
       <c r="E14" s="21" t="n"/>
       <c r="F14" s="21" t="n"/>
       <c r="G14" s="21" t="n"/>
-      <c r="H14" s="22" t="n"/>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A15" s="13" t="n"/>
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Veille informationnelle — Feedly. Documents : flux Feedly agrégeant IT-Connect, Sécurité Off, Veille Cyber N59 et Sécurité Informatique.</t>
+        </is>
+      </c>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="21" t="n"/>
       <c r="D15" s="21" t="n"/>
       <c r="E15" s="21" t="n"/>
       <c r="F15" s="21" t="n"/>
       <c r="G15" s="21" t="n"/>
-      <c r="H15" s="22" t="n"/>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A16" s="13" t="n"/>
@@ -1539,7 +1571,7 @@
     <row r="20" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Inventaire du parc informatique (préparation d'un déménagement) : recensement des postes, écrans, périphériques et consommables ; vérification de l'état de chaque équipement.</t>
+          <t>Inventaire du parc informatique — préparation d'un déménagement. Documents : fichier Excel d'inventaire (postes, écrans, périphériques, consommables, imprimantes) avec état de chaque équipement.</t>
         </is>
       </c>
       <c r="B20" s="11" t="n"/>
@@ -1557,7 +1589,7 @@
     <row r="21" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Suivi des tickets et incidents (Freshservice) : traitement d'un ticket de création de compte, priorisation des incidents selon leur gravité.</t>
+          <t>Suivi des tickets et incidents — Freshservice. Documents : ticket de création de compte suivi de bout en bout, notes de la réunion de priorisation des incidents.</t>
         </is>
       </c>
       <c r="B21" s="11" t="n"/>
@@ -1575,7 +1607,7 @@
     <row r="22" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Gestion d'un compte utilisateur (Microsoft 365) : création, affectation à un groupe, vérification des droits et accès.</t>
+          <t>Gestion d'un compte utilisateur — Microsoft 365. Documents : fiche de suivi de création de compte (affectation groupe, droits vérifiés).</t>
         </is>
       </c>
       <c r="B22" s="11" t="n"/>
@@ -1593,12 +1625,16 @@
     <row r="23" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>Infrastructure de supervision des serveurs (Hyper-V, Docker, Prometheus, Grafana, Windows Exporter, Alertmanager) : collecte de métriques, tableaux de bord, alertes automatiques par email, documentation technique.</t>
+          <t>Infrastructure de supervision des serveurs — Hyper-V, Docker, Prometheus, Grafana, Windows Exporter, Alertmanager. Documents : fichiers docker-compose.yml, règles d'alertes windows-alerts.yml, tableaux de bord Grafana, documentation technique complète.</t>
         </is>
       </c>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="21" t="n"/>
-      <c r="D23" s="21" t="n"/>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E23" s="21" t="n"/>
       <c r="F23" s="21" t="inlineStr">
         <is>
@@ -1611,7 +1647,7 @@
     <row r="24" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>Masterisation et déploiement via PXE : déploiement réseau d'une image système standardisée sur plusieurs postes.</t>
+          <t>Masterisation et déploiement via PXE. Documents : procédure de démarrage réseau (PXE), image système standardisée déployée.</t>
         </is>
       </c>
       <c r="B24" s="11" t="n"/>
@@ -1629,11 +1665,15 @@
     <row r="25" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>Masterisation d'un poste et création de compte (Windows 11, Microsoft 365) : préparation complète d'un poste pour un nouvel utilisateur.</t>
+          <t>Masterisation d'un poste et création de compte — Windows 11, Microsoft 365. Documents : poste déployé avec image préconfigurée, compte utilisateur créé et licencié.</t>
         </is>
       </c>
       <c r="B25" s="11" t="n"/>
-      <c r="C25" s="21" t="n"/>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D25" s="21" t="n"/>
       <c r="E25" s="21" t="n"/>
       <c r="F25" s="21" t="n"/>
@@ -1647,12 +1687,16 @@
     <row r="26" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>Supervision de disponibilité avec Uptime Kuma : sondes HTTPS, TCP, Ping et DNS sur le site web et les services réseau.</t>
+          <t>Supervision de disponibilité — Uptime Kuma. Documents : fichier docker-compose.yml, sondes HTTPS/TCP/Ping/DNS configurées, documentation technique.</t>
         </is>
       </c>
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E26" s="21" t="n"/>
       <c r="F26" s="21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ajout des missions ToolBox et Civray (E5 + fiche E6 n°2)
</commit_message>
<xml_diff>
--- a/assets/Tableau_E5_Kabir_AMOUSSA.xlsx
+++ b/assets/Tableau_E5_Kabir_AMOUSSA.xlsx
@@ -1525,9 +1525,17 @@
       </c>
     </row>
     <row r="16" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A16" s="13" t="n"/>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Clé USB bootable multi-OS de dépannage (Ventoy). Documents : clé Ventoy fonctionnelle, procédures rédigées pour MemTest86 et Kaspersky Rescue Disk.</t>
+        </is>
+      </c>
       <c r="B16" s="11" t="n"/>
-      <c r="C16" s="21" t="n"/>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D16" s="21" t="n"/>
       <c r="E16" s="21" t="n"/>
       <c r="F16" s="21" t="n"/>
@@ -1535,13 +1543,25 @@
       <c r="H16" s="22" t="n"/>
     </row>
     <row r="17" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A17" s="13" t="n"/>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Conception et déploiement du réseau de la médiathèque de Civray (MediaTek86). Documents : plan d'adressage, schémas réseau avant/après, configurations SW-Core et routeur WAN, captures des tests de connectivité, justifications techniques.</t>
+        </is>
+      </c>
       <c r="B17" s="11" t="n"/>
-      <c r="C17" s="21" t="n"/>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="D17" s="21" t="n"/>
       <c r="E17" s="21" t="n"/>
       <c r="F17" s="21" t="n"/>
-      <c r="G17" s="21" t="n"/>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H17" s="22" t="n"/>
     </row>
     <row r="18" ht="39.95" customFormat="1" customHeight="1" s="2">

</xml_diff>